<commit_message>
added code for Romania JobChanges- Partilly completed.
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Romania_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Romania_Regression_PK17.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="165">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -250,576 +250,1114 @@
     <t>Test1</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Sigurd Hackett' Employee:{undefined}TimeoutError: locator.click: Timeout 30000ms exceeded.
+    <t>10699818</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>880 Recruitment (Vofur Hagovi (10551546))</t>
+  </si>
+  <si>
+    <t>Romania</t>
+  </si>
+  <si>
+    <t>Bridgette</t>
+  </si>
+  <si>
+    <t>Aufderhar</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Automation Street Name</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>ABRUD</t>
+  </si>
+  <si>
+    <t>Alba</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t>automation@qe.com</t>
+  </si>
+  <si>
+    <t>New Hire</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Retail Assistant_NEW</t>
+  </si>
+  <si>
+    <t>Full Time</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>C - Regular labour contract (Romania Contract Types-Romania)@522303@DN - Daylight and Night hours (Romania Time Allocation-Romania)</t>
+  </si>
+  <si>
+    <t>5 Days</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Automation Comments here….</t>
+  </si>
+  <si>
+    <t>94 Retail Operatives</t>
+  </si>
+  <si>
+    <t>06 Menswear</t>
+  </si>
+  <si>
+    <t>Please select a Romania Pay Group</t>
+  </si>
+  <si>
+    <t>RO Monthly</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Choice A</t>
+  </si>
+  <si>
+    <t>ALBA</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Determined</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Personal Numeric Code (CNP)</t>
+  </si>
+  <si>
+    <t>1591231084975</t>
+  </si>
+  <si>
+    <t>01/01/2000</t>
+  </si>
+  <si>
+    <t>01/01/2040</t>
+  </si>
+  <si>
+    <t>Identity Card Number</t>
+  </si>
+  <si>
+    <t>Defaulted</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>01/03/1980</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Citizen (Romania)</t>
+  </si>
+  <si>
+    <t>ABN AMRO BANK ROMANIA</t>
+  </si>
+  <si>
+    <t>ABNA</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>1B31007593840000</t>
+  </si>
+  <si>
+    <t>RO49 AAAA 1B31 00759384 0000</t>
+  </si>
+  <si>
+    <t>Father's Name</t>
+  </si>
+  <si>
+    <t>AutoB</t>
+  </si>
+  <si>
+    <t>one fine</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'Sonny Jakubowski' Employee:{undefined}Error: [31mTimed out 5000ms waiting for [39m[2mexpect([22m[31mlocator[39m[2m).[22mtoBeVisible[2m()[22m
+Locator: locator('xpath=((//div[contains(text(),\'Awaiting Action\')]//ancestor::td//following-sibling::td)[3])[2]')
+Expected: visible
+Received: &lt;element(s) not found&gt;
 Call log:
-  [2m- waiting for locator('button:has-text("Submit")')[22m
-[2m  -   locator resolved to &lt;button type="button" title="Submit" class="WIWM WEDO WJ…&gt;…&lt;/button&gt;[22m
+  [2m- expect.toBeVisible with timeout 5000ms[22m
+[2m  - waiting for locator('xpath=((//div[contains(text(),\'Awaiting Action\')]//ancestor::td//following-sibling::td)[3])[2]')[22m
+</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>880 Store Management (Suvug Rozery (10629083))</t>
+  </si>
+  <si>
+    <t>Sonny</t>
+  </si>
+  <si>
+    <t>Jakubowski</t>
+  </si>
+  <si>
+    <t>Auto 29394639</t>
+  </si>
+  <si>
+    <t>Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>Part Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92 Retail Management </t>
+  </si>
+  <si>
+    <t>251 Management Retail</t>
+  </si>
+  <si>
+    <t>1680727103159</t>
+  </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>10699814</t>
+  </si>
+  <si>
+    <t>Sandra</t>
+  </si>
+  <si>
+    <t>Willms</t>
+  </si>
+  <si>
+    <t>1280128098445</t>
+  </si>
+  <si>
+    <t>Test4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'Mylene Lowe' Employee:{}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByLabel('My Tasks Items')[22m
+[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
 [2m  - attempting click action[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #1[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #2[22m
 [2m  -   waiting 20ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #3[22m
 [2m  -   waiting 100ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #4[22m
 [2m  -   waiting 100ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #5[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #6[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #7[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #8[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #9[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #10[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #11[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #12[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #13[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #14[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #15[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #16[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #17[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #18[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #19[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #20[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #21[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #22[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #23[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #24[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #25[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #26[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #27[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #28[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #29[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #30[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #31[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #32[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #33[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #34[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #35[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #36[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #37[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #38[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #39[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #40[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #41[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #42[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #43[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #44[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #45[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #46[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #47[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #48[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #49[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #50[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #51[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #52[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #53[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
 [2m  -   element is visible, enabled and stable[22m
 [2m  -   scrolling into view if needed[22m
 [2m  -   done scrolling[22m
-[2m  -   &lt;div class="WMT"&gt;…&lt;/div&gt; from &lt;div class="WAU WNT" data-automation-widget="wd-popup"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
 [2m  - retrying click action, attempt #54[22m
 [2m  -   waiting 500ms[22m
 [2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #55[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #56[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #57[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #58[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #59[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #60[22m
+[2m  -   waiting 500ms[22m
 </t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>880 Recruitment (Vofur Hagovi (10551546))</t>
-  </si>
-  <si>
-    <t>Romania</t>
-  </si>
-  <si>
-    <t>Sigurd</t>
-  </si>
-  <si>
-    <t>Hackett</t>
-  </si>
-  <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Automation Street Name</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>ABRUD</t>
-  </si>
-  <si>
-    <t>Alba</t>
-  </si>
-  <si>
-    <t>Street Address</t>
-  </si>
-  <si>
-    <t>automation@qe.com</t>
-  </si>
-  <si>
-    <t>New Hire</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Retail Assistant_NEW</t>
-  </si>
-  <si>
-    <t>Full Time</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>C - Regular labour contract (Romania Contract Types-Romania)@522303@DN - Daylight and Night hours (Romania Time Allocation-Romania)</t>
-  </si>
-  <si>
-    <t>5 Days</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Automation Comments here….</t>
-  </si>
-  <si>
-    <t>94 Retail Operatives</t>
-  </si>
-  <si>
-    <t>06 Menswear</t>
-  </si>
-  <si>
-    <t>Please select a Romania Pay Group</t>
-  </si>
-  <si>
-    <t>RO Monthly</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Choice A</t>
-  </si>
-  <si>
-    <t>ALBA</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Determined</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Personal Numeric Code (CNP)</t>
-  </si>
-  <si>
-    <t>1630206286772</t>
-  </si>
-  <si>
-    <t>01/01/2000</t>
-  </si>
-  <si>
-    <t>01/01/2040</t>
-  </si>
-  <si>
-    <t>Identity Card Number</t>
-  </si>
-  <si>
-    <t>Defaulted</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>01/03/1980</t>
-  </si>
-  <si>
-    <t>Single</t>
-  </si>
-  <si>
-    <t>Citizen (Romania)</t>
-  </si>
-  <si>
-    <t>ABN AMRO BANK ROMANIA</t>
-  </si>
-  <si>
-    <t>ABNA</t>
-  </si>
-  <si>
-    <t>Checking</t>
-  </si>
-  <si>
-    <t>1B31007593840000</t>
-  </si>
-  <si>
-    <t>RO49 AAAA 1B31 00759384 0000</t>
-  </si>
-  <si>
-    <t>Father's Name</t>
-  </si>
-  <si>
-    <t>AutoB</t>
-  </si>
-  <si>
-    <t>one fine</t>
-  </si>
-  <si>
-    <t>Test2</t>
-  </si>
-  <si>
-    <t>10699621</t>
-  </si>
-  <si>
-    <t>Passed</t>
-  </si>
-  <si>
-    <t>880 Store Management (Suvug Rozery (10629083))</t>
-  </si>
-  <si>
-    <t>Zackary</t>
-  </si>
-  <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>Auto 1757451</t>
-  </si>
-  <si>
-    <t>Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>Part Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92 Retail Management </t>
-  </si>
-  <si>
-    <t>251 Management Retail</t>
+    <t>Twila</t>
+  </si>
+  <si>
+    <t>Purdy</t>
+  </si>
+  <si>
+    <t>Auto 19435506</t>
+  </si>
+  <si>
+    <t>5140716248092</t>
+  </si>
+  <si>
+    <t>Test5</t>
+  </si>
+  <si>
+    <t>Test failed for 'Scot Barrows' Employee:{}Error: page.waitForTimeout: Target page, context or browser has been closed</t>
+  </si>
+  <si>
+    <t>Scot</t>
+  </si>
+  <si>
+    <t>Barrows</t>
+  </si>
+  <si>
+    <t>1710326367812</t>
+  </si>
+  <si>
+    <t>Test6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'Eveline Lowe' Employee:{}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByLabel('My Tasks Items')[22m
+[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #1[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #2[22m
+[2m  -   waiting 20ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #3[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #4[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #5[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #6[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #7[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #8[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #9[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #10[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #11[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #12[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #13[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #14[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #15[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #16[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #17[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #18[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #19[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #20[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #21[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #22[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #23[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #24[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #25[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #26[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #27[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #28[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #29[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #30[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #31[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #32[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #33[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #34[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #35[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #36[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #37[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #38[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #39[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #40[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #41[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #42[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #43[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #44[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #45[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #46[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #47[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #48[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #49[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #50[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #51[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #52[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #53[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #54[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #55[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #56[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #57[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #58[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div class="WJOP" data-automation-id="modalOverlay"&gt;…&lt;/div&gt; from &lt;div id="content-container"&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #59[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+</t>
+  </si>
+  <si>
+    <t>Eveline</t>
+  </si>
+  <si>
+    <t>Lowe</t>
+  </si>
+  <si>
+    <t>Auto 29987481</t>
+  </si>
+  <si>
+    <t>Fixed Term (Fixed Term)</t>
+  </si>
+  <si>
+    <t>5010204090714</t>
   </si>
 </sst>
 </file>
@@ -940,7 +1478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1051,6 +1589,12 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1332,7 +1876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CD3"/>
+  <dimension ref="A1:CD7"/>
   <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.81640625" style="1" customWidth="1"/>
@@ -1699,7 +2243,7 @@
       </c>
       <c r="K2" s="17">
         <f>TODAY()-100</f>
-        <v>45719</v>
+        <v>45731</v>
       </c>
       <c r="L2" s="14" t="s">
         <v>81</v>
@@ -1736,7 +2280,7 @@
       </c>
       <c r="W2" s="17">
         <f>TODAY()-100</f>
-        <v>45719</v>
+        <v>45731</v>
       </c>
       <c r="X2" s="16" t="s">
         <v>92</v>
@@ -1805,7 +2349,7 @@
         <v>1</v>
       </c>
       <c r="AT2" s="17">
-        <f t="shared" ref="AT2:AT3" si="0">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
+        <f t="shared" ref="AT2:AT7" si="0">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
         <v>NaN</v>
       </c>
       <c r="AU2" s="14" t="s">
@@ -1822,11 +2366,11 @@
       </c>
       <c r="AY2" s="17">
         <f>TODAY()-100</f>
-        <v>45719</v>
+        <v>45731</v>
       </c>
       <c r="AZ2" s="17">
         <f>TODAY()-100</f>
-        <v>45719</v>
+        <v>45731</v>
       </c>
       <c r="BA2" s="26" t="s">
         <v>100</v>
@@ -1854,7 +2398,7 @@
       </c>
       <c r="BI2" s="16">
         <f t="array" ref="BI2:BI3">_xlfn.RANDARRAY(2,1,123456,999999,TRUE)</f>
-        <v>723436</v>
+        <v>487904</v>
       </c>
       <c r="BJ2" s="19" t="s">
         <v>114</v>
@@ -1952,8 +2496,8 @@
         <v>85</v>
       </c>
       <c r="K3" s="34" t="str">
-        <f t="shared" ref="K3" si="1">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
-        <v>03/03/2025</v>
+        <f t="shared" ref="K3:K7" si="1">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
+        <v>15/03/2025</v>
       </c>
       <c r="L3" s="32" t="s">
         <v>81</v>
@@ -1989,8 +2533,8 @@
         <v>85</v>
       </c>
       <c r="W3" s="34" t="str">
-        <f t="shared" ref="W3" si="2">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
-        <v>03/03/2025</v>
+        <f t="shared" ref="W3:W7" si="2">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
+        <v>15/03/2025</v>
       </c>
       <c r="X3" s="16" t="s">
         <v>92</v>
@@ -2075,12 +2619,12 @@
         <v>111</v>
       </c>
       <c r="AY3" s="34" t="str">
-        <f t="shared" ref="AY3:AZ3" si="3">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
-        <v>03/03/2025</v>
+        <f t="shared" ref="AY3:AZ7" si="3">TEXT(TODAY()-100,"DD/MM/YYYY")</f>
+        <v>15/03/2025</v>
       </c>
       <c r="AZ3" s="34" t="str">
         <f t="shared" si="3"/>
-        <v>03/03/2025</v>
+        <v>15/03/2025</v>
       </c>
       <c r="BA3" s="37" t="str">
         <f>AH3</f>
@@ -2093,7 +2637,7 @@
         <v>112</v>
       </c>
       <c r="BD3" s="31" t="s">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="BE3" s="19" t="s">
         <v>114</v>
@@ -2108,7 +2652,7 @@
         <v>116</v>
       </c>
       <c r="BI3" s="16">
-        <v>972895</v>
+        <v>577003</v>
       </c>
       <c r="BJ3" s="19" t="s">
         <v>114</v>
@@ -2174,33 +2718,1060 @@
         <v>129</v>
       </c>
     </row>
+    <row r="4" ht="15.65" customHeight="1" spans="1:82" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="H4" s="16">
+        <v>720527700</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K4" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="M4" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="N4" s="16">
+        <v>1</v>
+      </c>
+      <c r="O4" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="P4" s="16">
+        <v>515100</v>
+      </c>
+      <c r="Q4" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="R4" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="S4" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="T4" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="U4" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="V4" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="W4" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y4" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z4" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA4" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB4" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC4" s="21">
+        <v>880</v>
+      </c>
+      <c r="AD4" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE4" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF4" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG4" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH4" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI4" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ4" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK4" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL4" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="AM4" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN4" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO4" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP4" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ4" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR4" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS4" s="16">
+        <v>1</v>
+      </c>
+      <c r="AT4" s="17">
+        <f t="shared" si="0"/>
+        <v>NaN</v>
+      </c>
+      <c r="AU4" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AV4" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW4" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="AX4" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="AY4" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="AZ4" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="BA4" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="BB4" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BC4" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="BD4" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="BE4" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BF4" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BG4" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH4" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="BI4" s="16">
+        <f t="array" ref="BI4:BI5">_xlfn.RANDARRAY(2,1,123456,999999,TRUE)</f>
+        <v>149064</v>
+      </c>
+      <c r="BJ4" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BK4" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BL4" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BM4" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BN4" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="BO4" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="BP4" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="BQ4" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="BR4" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="BS4" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="BT4" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="BU4" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="BV4" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="BW4" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="BX4" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="BY4" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="BZ4" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="CA4" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="CB4" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC4" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD4" s="29" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" ht="15.65" customHeight="1" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="H5" s="16">
+        <v>720527700</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K5" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="L5" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="M5" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="29">
+        <v>1</v>
+      </c>
+      <c r="O5" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" s="29">
+        <v>515100</v>
+      </c>
+      <c r="Q5" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="R5" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="S5" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="T5" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="U5" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="V5" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="W5" s="34" t="str">
+        <f t="shared" si="2"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="X5" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y5" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z5" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA5" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="AB5" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="AC5" s="21">
+        <v>880</v>
+      </c>
+      <c r="AD5" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE5" s="24">
+        <v>35</v>
+      </c>
+      <c r="AF5" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG5" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH5" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI5" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ5" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="AK5" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="AL5" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="AM5" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN5" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO5" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP5" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ5" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR5" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS5" s="16">
+        <v>2</v>
+      </c>
+      <c r="AT5" s="17">
+        <f t="shared" si="0"/>
+        <v>NaN</v>
+      </c>
+      <c r="AU5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AV5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW5" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="AX5" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="AY5" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="AZ5" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="BA5" s="37" t="str">
+        <f>AH5</f>
+        <v>N/A</v>
+      </c>
+      <c r="BB5" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BC5" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="BD5" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="BE5" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BF5" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BG5" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH5" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="BI5" s="16">
+        <v>763448</v>
+      </c>
+      <c r="BJ5" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BK5" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BL5" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BM5" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BN5" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="BO5" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="BP5" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="BQ5" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="BR5" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="BS5" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="BT5" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="BU5" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="BV5" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="BW5" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="BX5" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="BY5" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="BZ5" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="CA5" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="CB5" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC5" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD5" s="29" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" ht="15.65" customHeight="1" spans="1:82" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="H6" s="16">
+        <v>720527700</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K6" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="M6" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="N6" s="16">
+        <v>1</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="P6" s="16">
+        <v>515100</v>
+      </c>
+      <c r="Q6" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="R6" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="S6" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="T6" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="U6" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="V6" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="W6" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="X6" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y6" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z6" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA6" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB6" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC6" s="21">
+        <v>880</v>
+      </c>
+      <c r="AD6" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE6" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF6" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG6" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH6" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI6" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ6" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK6" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL6" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="AM6" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN6" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO6" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP6" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ6" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR6" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS6" s="16">
+        <v>1</v>
+      </c>
+      <c r="AT6" s="17">
+        <f t="shared" si="0"/>
+        <v>NaN</v>
+      </c>
+      <c r="AU6" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AV6" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW6" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="AX6" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="AY6" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="AZ6" s="17">
+        <f>TODAY()-100</f>
+        <v>45731</v>
+      </c>
+      <c r="BA6" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="BB6" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BC6" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="BD6" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="BE6" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BF6" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BG6" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH6" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="BI6" s="16">
+        <f t="array" ref="BI6:BI7">_xlfn.RANDARRAY(2,1,123456,999999,TRUE)</f>
+        <v>920186</v>
+      </c>
+      <c r="BJ6" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BK6" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BL6" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BM6" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BN6" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="BO6" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="BP6" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="BQ6" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="BR6" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="BS6" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="BT6" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="BU6" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="BV6" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="BW6" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="BX6" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="BY6" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="BZ6" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="CA6" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="CB6" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC6" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD6" s="29" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" ht="15.65" customHeight="1" spans="1:82" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="H7" s="16">
+        <v>720527700</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="L7" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="M7" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="N7" s="29">
+        <v>1</v>
+      </c>
+      <c r="O7" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="P7" s="29">
+        <v>515100</v>
+      </c>
+      <c r="Q7" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="R7" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="S7" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="T7" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="U7" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="V7" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="W7" s="34" t="str">
+        <f t="shared" si="2"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="X7" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y7" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="Z7" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA7" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="AB7" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="AC7" s="21">
+        <v>880</v>
+      </c>
+      <c r="AD7" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE7" s="24">
+        <v>35</v>
+      </c>
+      <c r="AF7" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG7" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH7" s="41">
+        <f>W7+364</f>
+        <v>46095</v>
+      </c>
+      <c r="AI7" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ7" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="AK7" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="AL7" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="AM7" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN7" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO7" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP7" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ7" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR7" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS7" s="16">
+        <v>2</v>
+      </c>
+      <c r="AT7" s="17">
+        <f t="shared" si="0"/>
+        <v>NaN</v>
+      </c>
+      <c r="AU7" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AV7" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW7" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="AX7" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="AY7" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="AZ7" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>15/03/2025</v>
+      </c>
+      <c r="BA7" s="41">
+        <f>AH7</f>
+        <v>46095</v>
+      </c>
+      <c r="BB7" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BC7" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="BD7" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="BE7" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BF7" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BG7" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="BH7" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="BI7" s="16">
+        <v>958457</v>
+      </c>
+      <c r="BJ7" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="BK7" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="BL7" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BM7" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BN7" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="BO7" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="BP7" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="BQ7" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="BR7" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="BS7" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="BT7" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="BU7" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="BV7" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="BW7" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="BX7" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="BY7" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="BZ7" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="CA7" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="CB7" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="CC7" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD7" s="29" t="s">
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX3">
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX7">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX7">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:J3">
       <formula1>INDIRECT(#REF!)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:J5">
       <formula1>INDIRECT(#REF!)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I7:J7">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J7">
+      <formula1>INDIRECT(#REF!)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S7">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V7">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X7">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="U2" r:id="rId1"/>
     <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U4" r:id="rId3"/>
+    <hyperlink ref="U5" r:id="rId4"/>
+    <hyperlink ref="U6" r:id="rId5"/>
+    <hyperlink ref="U7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>